<commit_message>
Manual orders (W- numbers, source/priority, edit/cancel), source filter + dashboard; sw v4
</commit_message>
<xml_diff>
--- a/Billing_Import_Template.xlsx
+++ b/Billing_Import_Template.xlsx
@@ -17,9 +17,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MM-YYYY"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD-MM-YYYY"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -75,14 +74,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +498,7 @@
           <t>EXAMPLE-2627/KDOP-3001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="7" t="n">
         <v>46313</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -519,7 +520,7 @@
           <t>EXAMPLE-2627/KDOP-3002</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="7" t="n">
         <v>46313</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -540,592 +541,592 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="n"/>
+      <c r="B4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="4" t="n"/>
+      <c r="B6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="4" t="n"/>
+      <c r="B7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="n"/>
+      <c r="B8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="4" t="n"/>
+      <c r="B9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="4" t="n"/>
+      <c r="B10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="n"/>
+      <c r="B11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="4" t="n"/>
+      <c r="B12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="4" t="n"/>
+      <c r="B13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="n"/>
+      <c r="B14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="n"/>
+      <c r="B15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="4" t="n"/>
+      <c r="B16" s="8" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="4" t="n"/>
+      <c r="B17" s="8" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="4" t="n"/>
+      <c r="B18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="4" t="n"/>
+      <c r="B19" s="8" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="4" t="n"/>
+      <c r="B20" s="8" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="4" t="n"/>
+      <c r="B21" s="8" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="4" t="n"/>
+      <c r="B22" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="4" t="n"/>
+      <c r="B23" s="8" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="4" t="n"/>
+      <c r="B24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="4" t="n"/>
+      <c r="B25" s="8" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="4" t="n"/>
+      <c r="B26" s="8" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="4" t="n"/>
+      <c r="B27" s="8" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="4" t="n"/>
+      <c r="B28" s="8" t="n"/>
     </row>
     <row r="29">
-      <c r="B29" s="4" t="n"/>
+      <c r="B29" s="8" t="n"/>
     </row>
     <row r="30">
-      <c r="B30" s="4" t="n"/>
+      <c r="B30" s="8" t="n"/>
     </row>
     <row r="31">
-      <c r="B31" s="4" t="n"/>
+      <c r="B31" s="8" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="4" t="n"/>
+      <c r="B32" s="8" t="n"/>
     </row>
     <row r="33">
-      <c r="B33" s="4" t="n"/>
+      <c r="B33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="B34" s="4" t="n"/>
+      <c r="B34" s="8" t="n"/>
     </row>
     <row r="35">
-      <c r="B35" s="4" t="n"/>
+      <c r="B35" s="8" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="4" t="n"/>
+      <c r="B36" s="8" t="n"/>
     </row>
     <row r="37">
-      <c r="B37" s="4" t="n"/>
+      <c r="B37" s="8" t="n"/>
     </row>
     <row r="38">
-      <c r="B38" s="4" t="n"/>
+      <c r="B38" s="8" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="4" t="n"/>
+      <c r="B39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="4" t="n"/>
+      <c r="B40" s="8" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="4" t="n"/>
+      <c r="B41" s="8" t="n"/>
     </row>
     <row r="42">
-      <c r="B42" s="4" t="n"/>
+      <c r="B42" s="8" t="n"/>
     </row>
     <row r="43">
-      <c r="B43" s="4" t="n"/>
+      <c r="B43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="4" t="n"/>
+      <c r="B44" s="8" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="4" t="n"/>
+      <c r="B45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="B46" s="4" t="n"/>
+      <c r="B46" s="8" t="n"/>
     </row>
     <row r="47">
-      <c r="B47" s="4" t="n"/>
+      <c r="B47" s="8" t="n"/>
     </row>
     <row r="48">
-      <c r="B48" s="4" t="n"/>
+      <c r="B48" s="8" t="n"/>
     </row>
     <row r="49">
-      <c r="B49" s="4" t="n"/>
+      <c r="B49" s="8" t="n"/>
     </row>
     <row r="50">
-      <c r="B50" s="4" t="n"/>
+      <c r="B50" s="8" t="n"/>
     </row>
     <row r="51">
-      <c r="B51" s="4" t="n"/>
+      <c r="B51" s="8" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="4" t="n"/>
+      <c r="B52" s="8" t="n"/>
     </row>
     <row r="53">
-      <c r="B53" s="4" t="n"/>
+      <c r="B53" s="8" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" s="4" t="n"/>
+      <c r="B54" s="8" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" s="4" t="n"/>
+      <c r="B55" s="8" t="n"/>
     </row>
     <row r="56">
-      <c r="B56" s="4" t="n"/>
+      <c r="B56" s="8" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" s="4" t="n"/>
+      <c r="B57" s="8" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" s="4" t="n"/>
+      <c r="B58" s="8" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" s="4" t="n"/>
+      <c r="B59" s="8" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="4" t="n"/>
+      <c r="B60" s="8" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" s="4" t="n"/>
+      <c r="B61" s="8" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" s="4" t="n"/>
+      <c r="B62" s="8" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" s="4" t="n"/>
+      <c r="B63" s="8" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" s="4" t="n"/>
+      <c r="B64" s="8" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" s="4" t="n"/>
+      <c r="B65" s="8" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="4" t="n"/>
+      <c r="B66" s="8" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" s="4" t="n"/>
+      <c r="B67" s="8" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="4" t="n"/>
+      <c r="B68" s="8" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" s="4" t="n"/>
+      <c r="B69" s="8" t="n"/>
     </row>
     <row r="70">
-      <c r="B70" s="4" t="n"/>
+      <c r="B70" s="8" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="4" t="n"/>
+      <c r="B71" s="8" t="n"/>
     </row>
     <row r="72">
-      <c r="B72" s="4" t="n"/>
+      <c r="B72" s="8" t="n"/>
     </row>
     <row r="73">
-      <c r="B73" s="4" t="n"/>
+      <c r="B73" s="8" t="n"/>
     </row>
     <row r="74">
-      <c r="B74" s="4" t="n"/>
+      <c r="B74" s="8" t="n"/>
     </row>
     <row r="75">
-      <c r="B75" s="4" t="n"/>
+      <c r="B75" s="8" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" s="4" t="n"/>
+      <c r="B76" s="8" t="n"/>
     </row>
     <row r="77">
-      <c r="B77" s="4" t="n"/>
+      <c r="B77" s="8" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="4" t="n"/>
+      <c r="B78" s="8" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" s="4" t="n"/>
+      <c r="B79" s="8" t="n"/>
     </row>
     <row r="80">
-      <c r="B80" s="4" t="n"/>
+      <c r="B80" s="8" t="n"/>
     </row>
     <row r="81">
-      <c r="B81" s="4" t="n"/>
+      <c r="B81" s="8" t="n"/>
     </row>
     <row r="82">
-      <c r="B82" s="4" t="n"/>
+      <c r="B82" s="8" t="n"/>
     </row>
     <row r="83">
-      <c r="B83" s="4" t="n"/>
+      <c r="B83" s="8" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" s="4" t="n"/>
+      <c r="B84" s="8" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" s="4" t="n"/>
+      <c r="B85" s="8" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" s="4" t="n"/>
+      <c r="B86" s="8" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="4" t="n"/>
+      <c r="B87" s="8" t="n"/>
     </row>
     <row r="88">
-      <c r="B88" s="4" t="n"/>
+      <c r="B88" s="8" t="n"/>
     </row>
     <row r="89">
-      <c r="B89" s="4" t="n"/>
+      <c r="B89" s="8" t="n"/>
     </row>
     <row r="90">
-      <c r="B90" s="4" t="n"/>
+      <c r="B90" s="8" t="n"/>
     </row>
     <row r="91">
-      <c r="B91" s="4" t="n"/>
+      <c r="B91" s="8" t="n"/>
     </row>
     <row r="92">
-      <c r="B92" s="4" t="n"/>
+      <c r="B92" s="8" t="n"/>
     </row>
     <row r="93">
-      <c r="B93" s="4" t="n"/>
+      <c r="B93" s="8" t="n"/>
     </row>
     <row r="94">
-      <c r="B94" s="4" t="n"/>
+      <c r="B94" s="8" t="n"/>
     </row>
     <row r="95">
-      <c r="B95" s="4" t="n"/>
+      <c r="B95" s="8" t="n"/>
     </row>
     <row r="96">
-      <c r="B96" s="4" t="n"/>
+      <c r="B96" s="8" t="n"/>
     </row>
     <row r="97">
-      <c r="B97" s="4" t="n"/>
+      <c r="B97" s="8" t="n"/>
     </row>
     <row r="98">
-      <c r="B98" s="4" t="n"/>
+      <c r="B98" s="8" t="n"/>
     </row>
     <row r="99">
-      <c r="B99" s="4" t="n"/>
+      <c r="B99" s="8" t="n"/>
     </row>
     <row r="100">
-      <c r="B100" s="4" t="n"/>
+      <c r="B100" s="8" t="n"/>
     </row>
     <row r="101">
-      <c r="B101" s="4" t="n"/>
+      <c r="B101" s="8" t="n"/>
     </row>
     <row r="102">
-      <c r="B102" s="4" t="n"/>
+      <c r="B102" s="8" t="n"/>
     </row>
     <row r="103">
-      <c r="B103" s="4" t="n"/>
+      <c r="B103" s="8" t="n"/>
     </row>
     <row r="104">
-      <c r="B104" s="4" t="n"/>
+      <c r="B104" s="8" t="n"/>
     </row>
     <row r="105">
-      <c r="B105" s="4" t="n"/>
+      <c r="B105" s="8" t="n"/>
     </row>
     <row r="106">
-      <c r="B106" s="4" t="n"/>
+      <c r="B106" s="8" t="n"/>
     </row>
     <row r="107">
-      <c r="B107" s="4" t="n"/>
+      <c r="B107" s="8" t="n"/>
     </row>
     <row r="108">
-      <c r="B108" s="4" t="n"/>
+      <c r="B108" s="8" t="n"/>
     </row>
     <row r="109">
-      <c r="B109" s="4" t="n"/>
+      <c r="B109" s="8" t="n"/>
     </row>
     <row r="110">
-      <c r="B110" s="4" t="n"/>
+      <c r="B110" s="8" t="n"/>
     </row>
     <row r="111">
-      <c r="B111" s="4" t="n"/>
+      <c r="B111" s="8" t="n"/>
     </row>
     <row r="112">
-      <c r="B112" s="4" t="n"/>
+      <c r="B112" s="8" t="n"/>
     </row>
     <row r="113">
-      <c r="B113" s="4" t="n"/>
+      <c r="B113" s="8" t="n"/>
     </row>
     <row r="114">
-      <c r="B114" s="4" t="n"/>
+      <c r="B114" s="8" t="n"/>
     </row>
     <row r="115">
-      <c r="B115" s="4" t="n"/>
+      <c r="B115" s="8" t="n"/>
     </row>
     <row r="116">
-      <c r="B116" s="4" t="n"/>
+      <c r="B116" s="8" t="n"/>
     </row>
     <row r="117">
-      <c r="B117" s="4" t="n"/>
+      <c r="B117" s="8" t="n"/>
     </row>
     <row r="118">
-      <c r="B118" s="4" t="n"/>
+      <c r="B118" s="8" t="n"/>
     </row>
     <row r="119">
-      <c r="B119" s="4" t="n"/>
+      <c r="B119" s="8" t="n"/>
     </row>
     <row r="120">
-      <c r="B120" s="4" t="n"/>
+      <c r="B120" s="8" t="n"/>
     </row>
     <row r="121">
-      <c r="B121" s="4" t="n"/>
+      <c r="B121" s="8" t="n"/>
     </row>
     <row r="122">
-      <c r="B122" s="4" t="n"/>
+      <c r="B122" s="8" t="n"/>
     </row>
     <row r="123">
-      <c r="B123" s="4" t="n"/>
+      <c r="B123" s="8" t="n"/>
     </row>
     <row r="124">
-      <c r="B124" s="4" t="n"/>
+      <c r="B124" s="8" t="n"/>
     </row>
     <row r="125">
-      <c r="B125" s="4" t="n"/>
+      <c r="B125" s="8" t="n"/>
     </row>
     <row r="126">
-      <c r="B126" s="4" t="n"/>
+      <c r="B126" s="8" t="n"/>
     </row>
     <row r="127">
-      <c r="B127" s="4" t="n"/>
+      <c r="B127" s="8" t="n"/>
     </row>
     <row r="128">
-      <c r="B128" s="4" t="n"/>
+      <c r="B128" s="8" t="n"/>
     </row>
     <row r="129">
-      <c r="B129" s="4" t="n"/>
+      <c r="B129" s="8" t="n"/>
     </row>
     <row r="130">
-      <c r="B130" s="4" t="n"/>
+      <c r="B130" s="8" t="n"/>
     </row>
     <row r="131">
-      <c r="B131" s="4" t="n"/>
+      <c r="B131" s="8" t="n"/>
     </row>
     <row r="132">
-      <c r="B132" s="4" t="n"/>
+      <c r="B132" s="8" t="n"/>
     </row>
     <row r="133">
-      <c r="B133" s="4" t="n"/>
+      <c r="B133" s="8" t="n"/>
     </row>
     <row r="134">
-      <c r="B134" s="4" t="n"/>
+      <c r="B134" s="8" t="n"/>
     </row>
     <row r="135">
-      <c r="B135" s="4" t="n"/>
+      <c r="B135" s="8" t="n"/>
     </row>
     <row r="136">
-      <c r="B136" s="4" t="n"/>
+      <c r="B136" s="8" t="n"/>
     </row>
     <row r="137">
-      <c r="B137" s="4" t="n"/>
+      <c r="B137" s="8" t="n"/>
     </row>
     <row r="138">
-      <c r="B138" s="4" t="n"/>
+      <c r="B138" s="8" t="n"/>
     </row>
     <row r="139">
-      <c r="B139" s="4" t="n"/>
+      <c r="B139" s="8" t="n"/>
     </row>
     <row r="140">
-      <c r="B140" s="4" t="n"/>
+      <c r="B140" s="8" t="n"/>
     </row>
     <row r="141">
-      <c r="B141" s="4" t="n"/>
+      <c r="B141" s="8" t="n"/>
     </row>
     <row r="142">
-      <c r="B142" s="4" t="n"/>
+      <c r="B142" s="8" t="n"/>
     </row>
     <row r="143">
-      <c r="B143" s="4" t="n"/>
+      <c r="B143" s="8" t="n"/>
     </row>
     <row r="144">
-      <c r="B144" s="4" t="n"/>
+      <c r="B144" s="8" t="n"/>
     </row>
     <row r="145">
-      <c r="B145" s="4" t="n"/>
+      <c r="B145" s="8" t="n"/>
     </row>
     <row r="146">
-      <c r="B146" s="4" t="n"/>
+      <c r="B146" s="8" t="n"/>
     </row>
     <row r="147">
-      <c r="B147" s="4" t="n"/>
+      <c r="B147" s="8" t="n"/>
     </row>
     <row r="148">
-      <c r="B148" s="4" t="n"/>
+      <c r="B148" s="8" t="n"/>
     </row>
     <row r="149">
-      <c r="B149" s="4" t="n"/>
+      <c r="B149" s="8" t="n"/>
     </row>
     <row r="150">
-      <c r="B150" s="4" t="n"/>
+      <c r="B150" s="8" t="n"/>
     </row>
     <row r="151">
-      <c r="B151" s="4" t="n"/>
+      <c r="B151" s="8" t="n"/>
     </row>
     <row r="152">
-      <c r="B152" s="4" t="n"/>
+      <c r="B152" s="8" t="n"/>
     </row>
     <row r="153">
-      <c r="B153" s="4" t="n"/>
+      <c r="B153" s="8" t="n"/>
     </row>
     <row r="154">
-      <c r="B154" s="4" t="n"/>
+      <c r="B154" s="8" t="n"/>
     </row>
     <row r="155">
-      <c r="B155" s="4" t="n"/>
+      <c r="B155" s="8" t="n"/>
     </row>
     <row r="156">
-      <c r="B156" s="4" t="n"/>
+      <c r="B156" s="8" t="n"/>
     </row>
     <row r="157">
-      <c r="B157" s="4" t="n"/>
+      <c r="B157" s="8" t="n"/>
     </row>
     <row r="158">
-      <c r="B158" s="4" t="n"/>
+      <c r="B158" s="8" t="n"/>
     </row>
     <row r="159">
-      <c r="B159" s="4" t="n"/>
+      <c r="B159" s="8" t="n"/>
     </row>
     <row r="160">
-      <c r="B160" s="4" t="n"/>
+      <c r="B160" s="8" t="n"/>
     </row>
     <row r="161">
-      <c r="B161" s="4" t="n"/>
+      <c r="B161" s="8" t="n"/>
     </row>
     <row r="162">
-      <c r="B162" s="4" t="n"/>
+      <c r="B162" s="8" t="n"/>
     </row>
     <row r="163">
-      <c r="B163" s="4" t="n"/>
+      <c r="B163" s="8" t="n"/>
     </row>
     <row r="164">
-      <c r="B164" s="4" t="n"/>
+      <c r="B164" s="8" t="n"/>
     </row>
     <row r="165">
-      <c r="B165" s="4" t="n"/>
+      <c r="B165" s="8" t="n"/>
     </row>
     <row r="166">
-      <c r="B166" s="4" t="n"/>
+      <c r="B166" s="8" t="n"/>
     </row>
     <row r="167">
-      <c r="B167" s="4" t="n"/>
+      <c r="B167" s="8" t="n"/>
     </row>
     <row r="168">
-      <c r="B168" s="4" t="n"/>
+      <c r="B168" s="8" t="n"/>
     </row>
     <row r="169">
-      <c r="B169" s="4" t="n"/>
+      <c r="B169" s="8" t="n"/>
     </row>
     <row r="170">
-      <c r="B170" s="4" t="n"/>
+      <c r="B170" s="8" t="n"/>
     </row>
     <row r="171">
-      <c r="B171" s="4" t="n"/>
+      <c r="B171" s="8" t="n"/>
     </row>
     <row r="172">
-      <c r="B172" s="4" t="n"/>
+      <c r="B172" s="8" t="n"/>
     </row>
     <row r="173">
-      <c r="B173" s="4" t="n"/>
+      <c r="B173" s="8" t="n"/>
     </row>
     <row r="174">
-      <c r="B174" s="4" t="n"/>
+      <c r="B174" s="8" t="n"/>
     </row>
     <row r="175">
-      <c r="B175" s="4" t="n"/>
+      <c r="B175" s="8" t="n"/>
     </row>
     <row r="176">
-      <c r="B176" s="4" t="n"/>
+      <c r="B176" s="8" t="n"/>
     </row>
     <row r="177">
-      <c r="B177" s="4" t="n"/>
+      <c r="B177" s="8" t="n"/>
     </row>
     <row r="178">
-      <c r="B178" s="4" t="n"/>
+      <c r="B178" s="8" t="n"/>
     </row>
     <row r="179">
-      <c r="B179" s="4" t="n"/>
+      <c r="B179" s="8" t="n"/>
     </row>
     <row r="180">
-      <c r="B180" s="4" t="n"/>
+      <c r="B180" s="8" t="n"/>
     </row>
     <row r="181">
-      <c r="B181" s="4" t="n"/>
+      <c r="B181" s="8" t="n"/>
     </row>
     <row r="182">
-      <c r="B182" s="4" t="n"/>
+      <c r="B182" s="8" t="n"/>
     </row>
     <row r="183">
-      <c r="B183" s="4" t="n"/>
+      <c r="B183" s="8" t="n"/>
     </row>
     <row r="184">
-      <c r="B184" s="4" t="n"/>
+      <c r="B184" s="8" t="n"/>
     </row>
     <row r="185">
-      <c r="B185" s="4" t="n"/>
+      <c r="B185" s="8" t="n"/>
     </row>
     <row r="186">
-      <c r="B186" s="4" t="n"/>
+      <c r="B186" s="8" t="n"/>
     </row>
     <row r="187">
-      <c r="B187" s="4" t="n"/>
+      <c r="B187" s="8" t="n"/>
     </row>
     <row r="188">
-      <c r="B188" s="4" t="n"/>
+      <c r="B188" s="8" t="n"/>
     </row>
     <row r="189">
-      <c r="B189" s="4" t="n"/>
+      <c r="B189" s="8" t="n"/>
     </row>
     <row r="190">
-      <c r="B190" s="4" t="n"/>
+      <c r="B190" s="8" t="n"/>
     </row>
     <row r="191">
-      <c r="B191" s="4" t="n"/>
+      <c r="B191" s="8" t="n"/>
     </row>
     <row r="192">
-      <c r="B192" s="4" t="n"/>
+      <c r="B192" s="8" t="n"/>
     </row>
     <row r="193">
-      <c r="B193" s="4" t="n"/>
+      <c r="B193" s="8" t="n"/>
     </row>
     <row r="194">
-      <c r="B194" s="4" t="n"/>
+      <c r="B194" s="8" t="n"/>
     </row>
     <row r="195">
-      <c r="B195" s="4" t="n"/>
+      <c r="B195" s="8" t="n"/>
     </row>
     <row r="196">
-      <c r="B196" s="4" t="n"/>
+      <c r="B196" s="8" t="n"/>
     </row>
     <row r="197">
-      <c r="B197" s="4" t="n"/>
+      <c r="B197" s="8" t="n"/>
     </row>
     <row r="198">
-      <c r="B198" s="4" t="n"/>
+      <c r="B198" s="8" t="n"/>
     </row>
     <row r="199">
-      <c r="B199" s="4" t="n"/>
+      <c r="B199" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1151,9 +1152,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1199,7 +1198,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Order Ref (optional): the Warehouse order no (e.g. 12 or W-12) or the Sales Tracker entry id. If given and found, it wins.</t>
+          <t xml:space="preserve">   Order Ref (optional): the order no shown in IM Warehouse (ST-175 for Sales Tracker orders, W-12 for orders added in the warehouse app). If given and found, it wins.</t>
         </is>
       </c>
     </row>
@@ -1217,9 +1216,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
@@ -1230,7 +1227,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> a) Order Ref matches a warehouse order no or Sales Tracker id: linked directly.</t>
+          <t xml:space="preserve"> a) Order Ref matches an order no (ST-.. / W-..) or Sales Tracker id: linked directly.</t>
         </is>
       </c>
     </row>

</xml_diff>